<commit_message>
Update Pires Lab website
</commit_message>
<xml_diff>
--- a/public/data/info.xlsx
+++ b/public/data/info.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\cisdeli\Purdue\CiampittiLab\ciampitti-lab.github.io\public\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pires\ciampitti-lab.github.io\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD7D56A7-DBBB-421C-9B21-E90A98FDE59D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{714C491D-1552-4706-AF24-4EC75CCAA910}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{680A29BD-E113-4DFE-A325-D924D35BBF8F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{680A29BD-E113-4DFE-A325-D924D35BBF8F}"/>
   </bookViews>
   <sheets>
     <sheet name="team" sheetId="1" r:id="rId1"/>
@@ -31,15 +31,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="137">
   <si>
     <t>role</t>
   </si>
@@ -59,36 +56,6 @@
     <t>name</t>
   </si>
   <si>
-    <t>Pedro Cisdeli</t>
-  </si>
-  <si>
-    <t>Gustavo Santiago</t>
-  </si>
-  <si>
-    <t>Leonardo Bosche</t>
-  </si>
-  <si>
-    <t>Natalia Volpato</t>
-  </si>
-  <si>
-    <t>Priscila Cano</t>
-  </si>
-  <si>
-    <t>Federico Gomez</t>
-  </si>
-  <si>
-    <t>German Mandrini</t>
-  </si>
-  <si>
-    <t>Thatiane Pereira</t>
-  </si>
-  <si>
-    <t>Franco Muriñigo</t>
-  </si>
-  <si>
-    <t>Ignacio Ciampitti</t>
-  </si>
-  <si>
     <t>id</t>
   </si>
   <si>
@@ -119,63 +86,15 @@
     <t>year</t>
   </si>
   <si>
-    <t>Postdoc</t>
-  </si>
-  <si>
-    <t>Biosystems Engineer researching digital agronomy. Works with sensors, web/mobile apps, computer vision, and AI for ag.</t>
-  </si>
-  <si>
-    <t>ML engineer bridging computer science and agronomy. Focused on computer vision, 3D reconstruction, data analysis and precision ag.</t>
-  </si>
-  <si>
-    <t>Focuses on crop modeling and data analysis. Background in agronomy with research on yield gaps, nutrient dynamics, and malting barley quality.</t>
-  </si>
-  <si>
-    <t>Works at the intersection of agronomy, data science, and economics. Focuses on crop modeling, big data, and decision tools to improve sustainability, profitability, and risk management in agriculture.</t>
-  </si>
-  <si>
-    <t>Lab Coordinator at Ciampitti Lab. Supports lab operations, chemical analysis, and data workflows, contributing to research and team coordination since 2022.</t>
-  </si>
-  <si>
-    <t>Field Coordinator at Ciampitti Lab. Oversees field operations, manages trial logistics, and ensures data collection quality across research sites.</t>
-  </si>
-  <si>
     <t>linkedin</t>
   </si>
   <si>
     <t>pfp_file_name</t>
   </si>
   <si>
-    <t>https://www.linkedin.com/in/ignaciociampitti/</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/in/pedro-cisdeli/</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/in/gustavo-nocera-santiago-00796616a/</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/in/leonardo-bosche/</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/in/natalia-volpato-3824a6150/</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/in/gmandrini/</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/in/priscilacano8/</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/in/thatiane-alves-pereira-13952719a/</t>
-  </si>
-  <si>
     <t>Faculty Advisor</t>
   </si>
   <si>
-    <t>Agronomy Professor and Principal Investigator. Leads research on digital ag, crop modeling, and remote sensing. Co-director of IDAAS at Purdue.</t>
-  </si>
-  <si>
     <t>category</t>
   </si>
   <si>
@@ -338,42 +257,6 @@
     <t>https://www.sciencedirect.com/science/article/abs/pii/S1161030124003496</t>
   </si>
   <si>
-    <t>ignacio_ciampitti.jpg</t>
-  </si>
-  <si>
-    <t>gustavo_santiago.jpg</t>
-  </si>
-  <si>
-    <t>thatiane_pereira.jpg</t>
-  </si>
-  <si>
-    <t>german_mandrini.png</t>
-  </si>
-  <si>
-    <t>leonardo_bosche.jpg</t>
-  </si>
-  <si>
-    <t>franco_murinigo.jpg</t>
-  </si>
-  <si>
-    <t>natalia_volpato.jpg</t>
-  </si>
-  <si>
-    <t>federico_gomez.jpg</t>
-  </si>
-  <si>
-    <t>priscila_cano.jpg</t>
-  </si>
-  <si>
-    <t>Agronomist developing decision support models for precision nitrogen management in corn. Integrates crop physiology, sensing technologies, and statistics to improve productivity while reducing environmental impact.</t>
-  </si>
-  <si>
-    <t>pedro_cisdeli.jpg</t>
-  </si>
-  <si>
-    <t>Combining expertise in agronomy, remote sensing &amp; geographic information systems, and economics. Current research efforts are directed toward the sustainable intensification of agricultural systems and digital agriculture.</t>
-  </si>
-  <si>
     <t>hello_world.md</t>
   </si>
   <si>
@@ -392,18 +275,6 @@
     <t>May 15, 2025</t>
   </si>
   <si>
-    <t>Agronomist researching sustainable corn-soybean systems, using digital tools to assess how crop rotation, cover crops, and nitrogen management impact soil health, environmental resilience, and overall farm productivity and profitability.</t>
-  </si>
-  <si>
-    <t>Roberto Romero</t>
-  </si>
-  <si>
-    <t>roberto_carlos.jpg</t>
-  </si>
-  <si>
-    <t>Passionate about agriculture, innovation, and exploration. Always eager to learn and take on new challenges in agronomy and agricultural advancement. Supports field operations through crop monitoring, data collection, and hands-on agricultural practices across research sites.</t>
-  </si>
-  <si>
     <t>Trends in agricultural technology: a review of US patents</t>
   </si>
   <si>
@@ -419,9 +290,6 @@
     <t>https://doi.org/10.1007/s11119-025-10257-x</t>
   </si>
   <si>
-    <t>https://www.linkedin.com/in/roberto-carlos-romero-palomeque-831917252?utm_source=share&amp;utm_campaign=share_via&amp;utm_content=profile&amp;utm_medium=ios_app</t>
-  </si>
-  <si>
     <t>Maize ear sensing for on-farm yield predictions</t>
   </si>
   <si>
@@ -458,65 +326,134 @@
     <t>Short series documenting Pedro Cisdeli's hands-on journey building ag-tech tools for Apple Vision Pro</t>
   </si>
   <si>
-    <t>Juan Fiore</t>
-  </si>
-  <si>
-    <t>jorge_jola.jpg</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/in/jjola-unal/</t>
-  </si>
-  <si>
-    <t>Jorge Jola</t>
-  </si>
-  <si>
-    <t>Undergraduate student in Agronomic Engineering at the National University of Colombia, with experience in agronomic data analysis. Skilled in statistics, Web applications, and the application of machine learning in agriculture.</t>
-  </si>
-  <si>
-    <t>Vlasis Mangidis</t>
-  </si>
-  <si>
-    <t>Data Scientist with a background in Agricultural Engineering and precision agriculture. Focuses on geospatial analytics and remote sensing using multispectral imagery. Experienced in Python, GIS, and database optimization to develop digital tools for vegetation analysis and decision support in agriculture.</t>
-  </si>
-  <si>
-    <t>vlasis_mangidis.jpg</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/in/vlasis-m-00537416b</t>
-  </si>
-  <si>
-    <t>Norman Menocal</t>
-  </si>
-  <si>
-    <t>norman_menocal.jpg</t>
-  </si>
-  <si>
-    <t>I am an agronomist interested in sustainable agriculture and the use of new technologies to improve the yield of agronomic crops. I have hands-on experience in fields crops, data collection, harvesting and pesticides applications, gained through academic projects and internship.</t>
-  </si>
-  <si>
-    <t>juan_fiore.png</t>
-  </si>
-  <si>
-    <t>Juan Douglas</t>
-  </si>
-  <si>
-    <t>juan_douglas.jpg</t>
-  </si>
-  <si>
-    <t>Agronomist graduated from the National University of Córdoba. Focused on digital agriculture with experience in Python and programming for agricultural applications. Areas of contribution include data management, digital tools, and the integration of technology into agricultural systems.</t>
-  </si>
-  <si>
-    <t>Agronomical Engineering undergraduate student from the national university of Colombia, passionate and skilled in fertigation, irrigation, soil physics, and the use of data in agriculture</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/in/juan-camilo-douglas-bolano-157646293/</t>
+    <t>Carlos Pires</t>
+  </si>
+  <si>
+    <t>Karen Cossi</t>
+  </si>
+  <si>
+    <t>Prashant Bhatt</t>
+  </si>
+  <si>
+    <t>Marcos Pedroso Menghini</t>
+  </si>
+  <si>
+    <t>Luis Fernando Bonini Pires</t>
+  </si>
+  <si>
+    <t>Maria Eduarda Boemo</t>
+  </si>
+  <si>
+    <t>Ellayna LaFond</t>
+  </si>
+  <si>
+    <t>Ezra Aberle</t>
+  </si>
+  <si>
+    <t>cossi_karen.jpg</t>
+  </si>
+  <si>
+    <t>lafond_ellayna.jpg</t>
+  </si>
+  <si>
+    <t>bhatt_prashant.jpg</t>
+  </si>
+  <si>
+    <t>pedroso_menghini_marcos.jpg</t>
+  </si>
+  <si>
+    <t>bonini_pires_luis fernando.jpg</t>
+  </si>
+  <si>
+    <t>boemo_maria.jpg</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/carlos-pires-75a953a6</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/karenck</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/prashant-bhatt-8ba7a3278</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/ellayna-lafond-83957823a</t>
+  </si>
+  <si>
+    <t>https://www.ndsu.edu/agriculture/ag-home/directory/ezra-aberle</t>
+  </si>
+  <si>
+    <t>https://br.linkedin.com/in/marcos-menghini-809620164</t>
+  </si>
+  <si>
+    <t>https://br.linkedin.com/in/maria-eduarda-boemo-312a70288</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ezra earned a B.S. in Animal Science and a M.S. in Crop Physiology and Production from Iowa State University. Currently he is pursuing his Ph.D. degree under the supervisor of Dr. Pires. </t>
+  </si>
+  <si>
+    <t>Prashant’s doctoral research focuses on soil dynamic properties under varying management intensities across North Dakota. His study emphasizes the long-term benefits of minimal soil disturbance and the response of different soil series to these management practices.</t>
+  </si>
+  <si>
+    <t>Ellayna's research examines the effects of land use—such as conventional tillage in agriculture (full till), conservation practices (minimal till or multi-cropping), and undisturbed systems (native prairies and grasslands)—on soil and water dynamics. Through this work, she aims to identify reliable indicators to define and predict soil health.</t>
+  </si>
+  <si>
+    <t>Luis is an intern student at the Pires Lab, taking part in several research projects, such as cover crop seeding and timing methods.</t>
+  </si>
+  <si>
+    <t>Maria Eduarda is now an student intern at the Pires Lab, contributing to several research projects.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marcos supports multiple research and extension projects throughout North Dakota as a student intern. </t>
+  </si>
+  <si>
+    <t>Dr. Pires' research focuses on regenerative agriculture, soil health and nutrient management for building resilient and sustainable agroecossystems.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Karen's research focusing on soil health under different soil management systems. Her research explores the long-term impacts of tillage practices, crop rotations and nitrogen sources on soil chemical, physical and biological indicator after 37 years of continuous soil building. </t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/luisfbpires/</t>
+  </si>
+  <si>
+    <t>pires_carlos.jpeg</t>
+  </si>
+  <si>
+    <t>current</t>
+  </si>
+  <si>
+    <t>Thassiany de Castro Alves</t>
+  </si>
+  <si>
+    <t>Artur Carmona</t>
+  </si>
+  <si>
+    <t>Marcos Centurion Gutierrez</t>
+  </si>
+  <si>
+    <t>centurion_gutierrez_marcos.jpg</t>
+  </si>
+  <si>
+    <t>de_casto_alves_thassiany.jpg</t>
+  </si>
+  <si>
+    <t>alumni</t>
+  </si>
+  <si>
+    <t>aberle_ezra.png</t>
+  </si>
+  <si>
+    <t>carmona_artur.jpg</t>
+  </si>
+  <si>
+    <t>group</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -554,12 +491,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -895,20 +829,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87EB64B1-8415-484E-B4A1-A632CC3BB222}">
-  <dimension ref="A1:F17"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="61.375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="182.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.5703125" customWidth="1"/>
+    <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.85546875" customWidth="1"/>
+    <col min="5" max="5" width="14.42578125" customWidth="1"/>
+    <col min="6" max="6" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B1" t="s">
         <v>5</v>
@@ -917,425 +851,350 @@
         <v>0</v>
       </c>
       <c r="D1" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="E1" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="G1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>96</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="D2" t="s">
-        <v>99</v>
+        <v>126</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>35</v>
+        <v>110</v>
       </c>
       <c r="F2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>123</v>
+      </c>
+      <c r="G2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>97</v>
       </c>
       <c r="C3" t="s">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>36</v>
+        <v>111</v>
       </c>
       <c r="F3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+        <v>124</v>
+      </c>
+      <c r="G3" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>98</v>
       </c>
       <c r="C4" t="s">
         <v>2</v>
       </c>
       <c r="D4" t="s">
-        <v>100</v>
-      </c>
-      <c r="E4" t="s">
-        <v>37</v>
+        <v>106</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>112</v>
       </c>
       <c r="F4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+        <v>118</v>
+      </c>
+      <c r="G4" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>102</v>
       </c>
       <c r="C5" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>38</v>
+        <v>113</v>
       </c>
       <c r="F5" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
+        <v>119</v>
+      </c>
+      <c r="G5" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>9</v>
+        <v>103</v>
       </c>
       <c r="C6" t="s">
         <v>2</v>
       </c>
       <c r="D6" t="s">
-        <v>105</v>
+        <v>134</v>
       </c>
       <c r="E6" t="s">
-        <v>39</v>
+        <v>114</v>
       </c>
       <c r="F6" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="7" spans="1:6">
+      <c r="G6" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>99</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="D7" t="s">
-        <v>106</v>
+        <v>107</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>115</v>
       </c>
       <c r="F7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
+        <v>122</v>
+      </c>
+      <c r="G7" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>100</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="D8" t="s">
-        <v>102</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>40</v>
+        <v>108</v>
+      </c>
+      <c r="E8" t="s">
+        <v>125</v>
       </c>
       <c r="F8" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="28.5">
+        <v>120</v>
+      </c>
+      <c r="G8" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>10</v>
+        <v>101</v>
       </c>
       <c r="C9" t="s">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="D9" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
+        <v>116</v>
+      </c>
+      <c r="F9" t="s">
+        <v>121</v>
+      </c>
+      <c r="G9" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>152</v>
+        <v>128</v>
       </c>
       <c r="C10" t="s">
         <v>3</v>
       </c>
       <c r="D10" t="s">
-        <v>153</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="F10" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
+        <v>132</v>
+      </c>
+      <c r="G10" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="C11" t="s">
         <v>3</v>
       </c>
       <c r="D11" t="s">
-        <v>151</v>
-      </c>
-      <c r="F11" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
+        <v>135</v>
+      </c>
+      <c r="G11" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>142</v>
+        <v>130</v>
       </c>
       <c r="C12" t="s">
         <v>3</v>
       </c>
       <c r="D12" t="s">
-        <v>140</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>141</v>
-      </c>
-      <c r="F12" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6">
-      <c r="A13">
-        <v>12</v>
-      </c>
-      <c r="B13" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13" t="s">
-        <v>3</v>
-      </c>
-      <c r="D13" t="s">
-        <v>104</v>
-      </c>
-      <c r="F13" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
-      <c r="A14">
-        <v>13</v>
-      </c>
-      <c r="B14" t="s">
-        <v>148</v>
-      </c>
-      <c r="C14" t="s">
-        <v>3</v>
-      </c>
-      <c r="D14" t="s">
-        <v>149</v>
-      </c>
-      <c r="F14" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="s">
-        <v>118</v>
-      </c>
-      <c r="C15" t="s">
-        <v>3</v>
-      </c>
-      <c r="D15" t="s">
-        <v>119</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="F15" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" t="s">
-        <v>13</v>
-      </c>
-      <c r="C16" t="s">
-        <v>3</v>
-      </c>
-      <c r="D16" t="s">
-        <v>101</v>
-      </c>
-      <c r="E16" t="s">
-        <v>42</v>
-      </c>
-      <c r="F16" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" t="s">
-        <v>144</v>
-      </c>
-      <c r="C17" t="s">
-        <v>3</v>
-      </c>
-      <c r="D17" t="s">
-        <v>146</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>147</v>
-      </c>
-      <c r="F17" t="s">
-        <v>145</v>
-      </c>
+        <v>131</v>
+      </c>
+      <c r="E12" s="1"/>
+      <c r="G12" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E14" s="1"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="E3" r:id="rId1" xr:uid="{AAA55F43-9F3C-40DB-9B47-46AAC432FF09}"/>
-    <hyperlink ref="E2" r:id="rId2" xr:uid="{A94255E5-8ECE-483E-BE8F-EE9B37DAE260}"/>
-    <hyperlink ref="E5" r:id="rId3" xr:uid="{F9808E56-71B8-4EF9-927B-9D68DAE7673D}"/>
-    <hyperlink ref="E8" r:id="rId4" xr:uid="{2A6658AF-7FC0-4FB5-9A94-14DD4D416741}"/>
-    <hyperlink ref="E15" r:id="rId5" xr:uid="{D4CFB1C7-1AE1-491B-850A-B6BFAE8BB6A7}"/>
-    <hyperlink ref="E12" r:id="rId6" tooltip="https://www.linkedin.com/in/jjola-unal/" xr:uid="{9B18B642-568C-42D5-8EB7-C9BF52A122A6}"/>
-    <hyperlink ref="E17" r:id="rId7" xr:uid="{83DA2968-3BAC-44C7-87DD-D7D2815CABF1}"/>
-    <hyperlink ref="E10" r:id="rId8" xr:uid="{C20D33EE-D7E5-4CF8-918D-658532FE0616}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8353AB8B-5FB3-4C2E-B56B-5EAF5DE5DE00}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="11.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C1" t="s">
-        <v>131</v>
+        <v>88</v>
       </c>
       <c r="D1" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="E1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" t="s">
         <v>19</v>
       </c>
-      <c r="F1" t="s">
-        <v>45</v>
-      </c>
       <c r="G1" t="s">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="H1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>114</v>
+        <v>76</v>
       </c>
       <c r="C2" t="s">
-        <v>132</v>
+        <v>89</v>
       </c>
       <c r="D2" t="s">
-        <v>113</v>
+        <v>75</v>
       </c>
       <c r="E2" t="s">
-        <v>116</v>
+        <v>78</v>
       </c>
       <c r="F2" t="s">
-        <v>115</v>
+        <v>77</v>
       </c>
       <c r="G2" t="s">
-        <v>111</v>
+        <v>73</v>
       </c>
       <c r="H2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>137</v>
+        <v>94</v>
       </c>
       <c r="C3" t="s">
-        <v>133</v>
+        <v>90</v>
       </c>
       <c r="D3" t="s">
-        <v>138</v>
+        <v>95</v>
       </c>
       <c r="E3" t="s">
-        <v>134</v>
+        <v>91</v>
       </c>
       <c r="F3" t="s">
-        <v>115</v>
+        <v>77</v>
       </c>
       <c r="G3" t="s">
-        <v>135</v>
+        <v>92</v>
       </c>
       <c r="H3" t="s">
-        <v>136</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>
@@ -1346,328 +1205,330 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA036B15-B04C-4846-822B-68722C1605FF}">
   <dimension ref="A1:G14"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="2" max="2" width="18.42578125" customWidth="1"/>
+    <col min="3" max="3" width="23.140625" customWidth="1"/>
     <col min="4" max="4" width="30" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="C1" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="D1" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="E1" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="F1" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="G1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>47</v>
+        <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="E2">
         <v>2025</v>
       </c>
       <c r="F2" t="s">
-        <v>51</v>
+        <v>25</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="C3" t="s">
-        <v>53</v>
+        <v>27</v>
       </c>
       <c r="D3" t="s">
-        <v>54</v>
+        <v>28</v>
       </c>
       <c r="E3">
         <v>2025</v>
       </c>
       <c r="F3" t="s">
-        <v>55</v>
+        <v>29</v>
       </c>
       <c r="G3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>57</v>
+        <v>31</v>
       </c>
       <c r="C4" t="s">
-        <v>58</v>
+        <v>32</v>
       </c>
       <c r="D4" t="s">
-        <v>59</v>
+        <v>33</v>
       </c>
       <c r="E4">
         <v>2025</v>
       </c>
       <c r="F4" t="s">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="C5" t="s">
-        <v>63</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>59</v>
+        <v>33</v>
       </c>
       <c r="E5">
         <v>2025</v>
       </c>
       <c r="F5" t="s">
-        <v>64</v>
+        <v>38</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>66</v>
+        <v>40</v>
       </c>
       <c r="C6" t="s">
-        <v>67</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s">
-        <v>69</v>
+        <v>43</v>
       </c>
       <c r="E6">
         <v>2025</v>
       </c>
       <c r="F6" t="s">
-        <v>68</v>
+        <v>42</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>72</v>
+        <v>46</v>
       </c>
       <c r="C7" t="s">
-        <v>71</v>
+        <v>45</v>
       </c>
       <c r="D7" t="s">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="E7">
         <v>2025</v>
       </c>
       <c r="F7" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>76</v>
+        <v>50</v>
       </c>
       <c r="C8" t="s">
-        <v>77</v>
+        <v>51</v>
       </c>
       <c r="D8" t="s">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="E8">
         <v>2025</v>
       </c>
       <c r="F8" t="s">
-        <v>78</v>
+        <v>52</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>80</v>
+        <v>54</v>
       </c>
       <c r="C9" t="s">
-        <v>81</v>
+        <v>55</v>
       </c>
       <c r="D9" t="s">
-        <v>82</v>
+        <v>56</v>
       </c>
       <c r="E9">
         <v>2025</v>
       </c>
       <c r="F9" t="s">
-        <v>84</v>
+        <v>58</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>85</v>
+        <v>59</v>
       </c>
       <c r="C10" t="s">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>87</v>
+        <v>61</v>
       </c>
       <c r="E10">
         <v>2025</v>
       </c>
       <c r="F10" t="s">
-        <v>98</v>
+        <v>72</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>88</v>
+        <v>62</v>
       </c>
       <c r="C11" t="s">
-        <v>89</v>
+        <v>63</v>
       </c>
       <c r="D11" t="s">
-        <v>82</v>
+        <v>56</v>
       </c>
       <c r="E11">
         <v>2025</v>
       </c>
       <c r="F11" t="s">
-        <v>96</v>
+        <v>70</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>90</v>
+        <v>64</v>
       </c>
       <c r="C12" t="s">
-        <v>91</v>
+        <v>65</v>
       </c>
       <c r="D12" t="s">
-        <v>92</v>
+        <v>66</v>
       </c>
       <c r="E12">
         <v>2025</v>
       </c>
       <c r="F12" t="s">
-        <v>94</v>
+        <v>68</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>121</v>
+        <v>79</v>
       </c>
       <c r="C13" t="s">
-        <v>122</v>
+        <v>80</v>
       </c>
       <c r="D13" t="s">
-        <v>123</v>
+        <v>81</v>
       </c>
       <c r="E13">
         <v>2025</v>
       </c>
       <c r="F13" t="s">
-        <v>124</v>
+        <v>82</v>
       </c>
       <c r="G13" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>127</v>
+        <v>84</v>
       </c>
       <c r="C14" t="s">
-        <v>128</v>
+        <v>85</v>
       </c>
       <c r="D14" t="s">
-        <v>130</v>
+        <v>87</v>
       </c>
       <c r="E14">
         <v>2025</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>129</v>
+        <v>86</v>
       </c>
       <c r="G14" s="1"/>
     </row>

</xml_diff>

<commit_message>
update colors and members
</commit_message>
<xml_diff>
--- a/public/data/info.xlsx
+++ b/public/data/info.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pires\ciampitti-lab.github.io\public\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13BEAF40-796D-4B37-A40C-2DD1707B24FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43065FA5-436A-4C8B-8501-B5B44ACC1125}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{680A29BD-E113-4DFE-A325-D924D35BBF8F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="139">
   <si>
     <t>role</t>
   </si>
@@ -398,9 +398,6 @@
     <t>Luis is an intern student at the Pires Lab, taking part in several research projects, such as cover crop seeding and timing methods.</t>
   </si>
   <si>
-    <t>Maria Eduarda is now an student intern at the Pires Lab, contributing to several research projects.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Marcos supports multiple research and extension projects throughout North Dakota as a student intern. </t>
   </si>
   <si>
@@ -447,13 +444,22 @@
   </si>
   <si>
     <t>Ellayna's research examines the effects of land use on soil and water dynamics. Through this work, she aims to identify reliable indicators to define and predict soil health.</t>
+  </si>
+  <si>
+    <t>Thassiany is conducting part of her doctoral research as a visiting scholar working on the project “Indicators of Soil Health under Different Long-Term Agricultural Practices”.</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/thassiany-de-castro-alves-13a148346/</t>
+  </si>
+  <si>
+    <t>Maria Eduarda is an student intern at the Pires Lab, contributing to several research projects.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -468,6 +474,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -491,9 +503,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -860,7 +873,7 @@
         <v>4</v>
       </c>
       <c r="G1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -874,16 +887,16 @@
         <v>18</v>
       </c>
       <c r="D2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>110</v>
       </c>
       <c r="F2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -903,10 +916,10 @@
         <v>111</v>
       </c>
       <c r="F3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -929,7 +942,7 @@
         <v>118</v>
       </c>
       <c r="G4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -949,10 +962,10 @@
         <v>113</v>
       </c>
       <c r="F5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -966,7 +979,7 @@
         <v>2</v>
       </c>
       <c r="D6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E6" t="s">
         <v>114</v>
@@ -975,7 +988,7 @@
         <v>117</v>
       </c>
       <c r="G6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -995,10 +1008,10 @@
         <v>115</v>
       </c>
       <c r="F7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1015,13 +1028,13 @@
         <v>108</v>
       </c>
       <c r="E8" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F8" t="s">
         <v>119</v>
       </c>
       <c r="G8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -1041,27 +1054,33 @@
         <v>116</v>
       </c>
       <c r="F9" t="s">
-        <v>120</v>
+        <v>138</v>
       </c>
       <c r="G9" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C10" t="s">
         <v>3</v>
       </c>
       <c r="D10" t="s">
-        <v>130</v>
+        <v>129</v>
+      </c>
+      <c r="E10" t="s">
+        <v>137</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>136</v>
       </c>
       <c r="G10" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -1069,16 +1088,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C11" t="s">
         <v>3</v>
       </c>
       <c r="D11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1086,17 +1105,17 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C12" t="s">
         <v>3</v>
       </c>
       <c r="D12" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E12" s="1"/>
       <c r="G12" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>